<commit_message>
Deploy Shopify Catalog Audits & Tracker (2026-10-28 18:53:43)
</commit_message>
<xml_diff>
--- a/crowcanyonhome/crowcanyonhome_5_upgraded_products.xlsx
+++ b/crowcanyonhome/crowcanyonhome_5_upgraded_products.xlsx
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -160,6 +160,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -531,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -570,35 +571,45 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Current Word Count</t>
+          <t>Feed Word Count (Shopify API)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Live Storefront Words (Theme)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Feed vs Theme Diagnostic</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Upgraded Description (Clean Readable Text + Specs)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Current Alt Text</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Upgraded Image Alt Text</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Upgraded Google Shopping Category</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Upgraded Smart Tags</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Live Product URL</t>
         </is>
@@ -628,7 +639,15 @@
       <c r="E2" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="n">
+        <v>127</v>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Feed vs Theme Disconnect (Theme renders copy, but raw API feed is 0w)</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>The Replacement Seal for #55 Salt &amp; Pepper Shakers by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
 Key Features &amp; Highlights
@@ -640,27 +659,27 @@
 Material / BuildHeirloom-Grade Materials with Hand-Finished DetailingApplicationDaily Residential &amp; Commercial Architectural UseCare &amp; MaintenanceWipe clean with soft damp cloth; food-safe / non-porousBrand OriginCrowcanyonhome (United States)Design StandardTimeless Modern Functionalism</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>Replacement Seal for #55 Salt &amp; Pepper Shakers - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Furniture</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="L2" s="10" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="M2" s="10" t="inlineStr">
         <is>
           <t>https://crowcanyonhome.com/products/replacement-seal-for-55-salt-pepper-shakers</t>
         </is>
@@ -690,7 +709,15 @@
       <c r="E3" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Feed vs Theme Disconnect (Theme renders copy, but raw API feed is 0w)</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>The Replacement Lids for the #102 Storage Bowls by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
 Key Features &amp; Highlights
@@ -702,27 +729,27 @@
 Material / BuildHeirloom-Grade Materials with Hand-Finished DetailingApplicationDaily Residential &amp; Commercial Architectural UseCare &amp; MaintenanceWipe clean with soft damp cloth; food-safe / non-porousBrand OriginCrowcanyonhome (United States)Design StandardTimeless Modern Functionalism</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Replacement Lids for the #102 Storage Bowls - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="K3" s="9" t="inlineStr">
+      <c r="M3" s="10" t="inlineStr">
         <is>
           <t>https://crowcanyonhome.com/products/replacement-lids-for-the-102-storage-bowls</t>
         </is>
@@ -752,7 +779,15 @@
       <c r="E4" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="7" t="n">
+        <v>153</v>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Standard Catalog Item</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>The Catalina Soy Candle 9 oz Mug by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
 Key Features &amp; Highlights
@@ -764,27 +799,27 @@
 Material / BuildHeirloom-Grade Materials with Hand-Finished DetailingApplicationDaily Residential &amp; Commercial Architectural UseCare &amp; MaintenanceWipe clean with soft damp cloth; food-safe / non-porousBrand OriginCrowcanyonhome (United States)Design StandardTimeless Modern Functionalism</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>Catalina Soy Candle 9 oz Mug - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="L4" s="10" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="M4" s="10" t="inlineStr">
         <is>
           <t>https://crowcanyonhome.com/products/catalina-soy-candle-9-oz-mug</t>
         </is>
@@ -814,7 +849,15 @@
       <c r="E5" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="7" t="n">
+        <v>170</v>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Standard Catalog Item</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>The Stinson Speckle 12 oz Mugs, Set of 4 by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
 Key Features &amp; Highlights
@@ -826,27 +869,27 @@
 Material / BuildHeirloom-Grade Materials with Hand-Finished DetailingApplicationDaily Residential &amp; Commercial Architectural UseCare &amp; MaintenanceWipe clean with soft damp cloth; food-safe / non-porousBrand OriginCrowcanyonhome (United States)Design StandardTimeless Modern Functionalism</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>Stinson Speckle 12 oz Mugs, Set of 4 - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="L5" s="10" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="K5" s="9" t="inlineStr">
+      <c r="M5" s="10" t="inlineStr">
         <is>
           <t>https://crowcanyonhome.com/products/cch-stinson-12-mugs</t>
         </is>
@@ -876,7 +919,15 @@
       <c r="E6" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="7" t="n">
+        <v>160</v>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Standard Catalog Item</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>The Vintage Dinner Plates, Set of 4 by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.
 Key Features &amp; Highlights
@@ -888,27 +939,27 @@
 Material / BuildHeirloom-Grade Materials with Hand-Finished DetailingApplicationDaily Residential &amp; Commercial Architectural UseCare &amp; MaintenanceWipe clean with soft damp cloth; food-safe / non-porousBrand OriginCrowcanyonhome (United States)Design StandardTimeless Modern Functionalism</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>Missing / Empty (Not Indexed)</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="J6" s="7" t="inlineStr">
         <is>
           <t>Vintage Dinner Plates, Set of 4 - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="L6" s="10" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="K6" s="9" t="inlineStr">
+      <c r="M6" s="10" t="inlineStr">
         <is>
           <t>https://crowcanyonhome.com/products/cch-vintage-dinner-plates</t>
         </is>
@@ -967,164 +1018,164 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Handle</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Body (HTML)</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Product Category</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Option1 Name</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Option1 Value</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Variant SKU</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="L1" s="11" t="inlineStr">
         <is>
           <t>Variant Grams</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="M1" s="11" t="inlineStr">
         <is>
           <t>Variant Inventory Tracker</t>
         </is>
       </c>
-      <c r="N1" s="10" t="inlineStr">
+      <c r="N1" s="11" t="inlineStr">
         <is>
           <t>Variant Inventory Qty</t>
         </is>
       </c>
-      <c r="O1" s="10" t="inlineStr">
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>Variant Inventory Policy</t>
         </is>
       </c>
-      <c r="P1" s="10" t="inlineStr">
+      <c r="P1" s="11" t="inlineStr">
         <is>
           <t>Variant Fulfillment Service</t>
         </is>
       </c>
-      <c r="Q1" s="10" t="inlineStr">
+      <c r="Q1" s="11" t="inlineStr">
         <is>
           <t>Variant Price</t>
         </is>
       </c>
-      <c r="R1" s="10" t="inlineStr">
+      <c r="R1" s="11" t="inlineStr">
         <is>
           <t>Variant Compare At Price</t>
         </is>
       </c>
-      <c r="S1" s="10" t="inlineStr">
+      <c r="S1" s="11" t="inlineStr">
         <is>
           <t>Variant Requires Shipping</t>
         </is>
       </c>
-      <c r="T1" s="10" t="inlineStr">
+      <c r="T1" s="11" t="inlineStr">
         <is>
           <t>Variant Taxable</t>
         </is>
       </c>
-      <c r="U1" s="10" t="inlineStr">
+      <c r="U1" s="11" t="inlineStr">
         <is>
           <t>Variant Barcode</t>
         </is>
       </c>
-      <c r="V1" s="10" t="inlineStr">
+      <c r="V1" s="11" t="inlineStr">
         <is>
           <t>Image Src</t>
         </is>
       </c>
-      <c r="W1" s="10" t="inlineStr">
+      <c r="W1" s="11" t="inlineStr">
         <is>
           <t>Image Position</t>
         </is>
       </c>
-      <c r="X1" s="10" t="inlineStr">
+      <c r="X1" s="11" t="inlineStr">
         <is>
           <t>Image Alt Text</t>
         </is>
       </c>
-      <c r="Y1" s="10" t="inlineStr">
+      <c r="Y1" s="11" t="inlineStr">
         <is>
           <t>Gift Card</t>
         </is>
       </c>
-      <c r="Z1" s="10" t="inlineStr">
+      <c r="Z1" s="11" t="inlineStr">
         <is>
           <t>SEO Title</t>
         </is>
       </c>
-      <c r="AA1" s="10" t="inlineStr">
+      <c r="AA1" s="11" t="inlineStr">
         <is>
           <t>SEO Description</t>
         </is>
       </c>
-      <c r="AB1" s="10" t="inlineStr">
+      <c r="AB1" s="11" t="inlineStr">
         <is>
           <t>Google Shopping / Google Product Category</t>
         </is>
       </c>
-      <c r="AC1" s="10" t="inlineStr">
+      <c r="AC1" s="11" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>replacement-seal-for-55-salt-pepper-shakers</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Replacement Seal for #55 Salt &amp; Pepper Shakers | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>&lt;p&gt;The &lt;strong&gt;Replacement Seal for #55 Salt &amp; Pepper Shakers&lt;/strong&gt; by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
 &lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
@@ -1139,141 +1190,141 @@
 &lt;/table&gt;</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Crowcanyonhome</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Furniture</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Furniture</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="H2" s="11" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I2" s="11" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J2" s="11" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K2" s="11" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>REPLACEMENT-SEAL-FOR-FIXED</t>
         </is>
       </c>
-      <c r="L2" s="11" t="inlineStr">
+      <c r="L2" s="12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M2" s="11" t="inlineStr">
+      <c r="M2" s="12" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N2" s="11" t="inlineStr">
+      <c r="N2" s="12" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O2" s="11" t="inlineStr">
+      <c r="O2" s="12" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P2" s="11" t="inlineStr">
+      <c r="P2" s="12" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q2" s="11" t="inlineStr">
+      <c r="Q2" s="12" t="inlineStr">
         <is>
           <t>5.00</t>
         </is>
       </c>
-      <c r="R2" s="11" t="inlineStr"/>
-      <c r="S2" s="11" t="inlineStr">
+      <c r="R2" s="12" t="inlineStr"/>
+      <c r="S2" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T2" s="11" t="inlineStr">
+      <c r="T2" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U2" s="11" t="inlineStr"/>
-      <c r="V2" s="11" t="inlineStr">
+      <c r="U2" s="12" t="inlineStr"/>
+      <c r="V2" s="12" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0068/3730/5397/files/D55-WEBBC_BLM.png?v=1790220345</t>
         </is>
       </c>
-      <c r="W2" s="11" t="inlineStr">
+      <c r="W2" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X2" s="11" t="inlineStr">
+      <c r="X2" s="12" t="inlineStr">
         <is>
           <t>Replacement Seal for #55 Salt &amp; Pepper Shakers - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="Y2" s="11" t="inlineStr">
+      <c r="Y2" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z2" s="11" t="inlineStr">
+      <c r="Z2" s="12" t="inlineStr">
         <is>
           <t>Replacement Seal for #55 Salt &amp; Pepper Shakers | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="AA2" s="11" t="inlineStr">
+      <c r="AA2" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">The  Replacement Seal for #55 Salt &amp; Pepper Shakers  by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. </t>
         </is>
       </c>
-      <c r="AB2" s="11" t="inlineStr">
+      <c r="AB2" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Furniture</t>
         </is>
       </c>
-      <c r="AC2" s="11" t="inlineStr">
+      <c r="AC2" s="12" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>replacement-lids-for-the-102-storage-bowls</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Replacement Lids for the #102 Storage Bowls | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>&lt;p&gt;The &lt;strong&gt;Replacement Lids for the #102 Storage Bowls&lt;/strong&gt; by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
 &lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
@@ -1288,141 +1339,141 @@
 &lt;/table&gt;</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Crowcanyonhome</t>
         </is>
       </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="12" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="H3" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="I3" s="12" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="J3" s="12" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K3" s="11" t="inlineStr">
+      <c r="K3" s="12" t="inlineStr">
         <is>
           <t>REPLACEMENT-LIDS-FOR-FIXED</t>
         </is>
       </c>
-      <c r="L3" s="11" t="inlineStr">
+      <c r="L3" s="12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M3" s="11" t="inlineStr">
+      <c r="M3" s="12" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N3" s="11" t="inlineStr">
+      <c r="N3" s="12" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O3" s="11" t="inlineStr">
+      <c r="O3" s="12" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P3" s="11" t="inlineStr">
+      <c r="P3" s="12" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q3" s="11" t="inlineStr">
+      <c r="Q3" s="12" t="inlineStr">
         <is>
           <t>5.00</t>
         </is>
       </c>
-      <c r="R3" s="11" t="inlineStr"/>
-      <c r="S3" s="11" t="inlineStr">
+      <c r="R3" s="12" t="inlineStr"/>
+      <c r="S3" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T3" s="11" t="inlineStr">
+      <c r="T3" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U3" s="11" t="inlineStr"/>
-      <c r="V3" s="11" t="inlineStr">
+      <c r="U3" s="12" t="inlineStr"/>
+      <c r="V3" s="12" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0068/3730/5397/files/cc_B81A0304_C102__16644.1713295343_1.webp?v=1790217105</t>
         </is>
       </c>
-      <c r="W3" s="11" t="inlineStr">
+      <c r="W3" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X3" s="11" t="inlineStr">
+      <c r="X3" s="12" t="inlineStr">
         <is>
           <t>Replacement Lids for the #102 Storage Bowls - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="Y3" s="11" t="inlineStr">
+      <c r="Y3" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z3" s="11" t="inlineStr">
+      <c r="Z3" s="12" t="inlineStr">
         <is>
           <t>Replacement Lids for the #102 Storage Bowls | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="AA3" s="11" t="inlineStr">
+      <c r="AA3" s="12" t="inlineStr">
         <is>
           <t>The  Replacement Lids for the #102 Storage Bowls  by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Tho</t>
         </is>
       </c>
-      <c r="AB3" s="11" t="inlineStr">
+      <c r="AB3" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="AC3" s="11" t="inlineStr">
+      <c r="AC3" s="12" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>catalina-soy-candle-9-oz-mug</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Catalina Soy Candle 9 oz Mug | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>&lt;p&gt;The &lt;strong&gt;Catalina Soy Candle 9 oz Mug&lt;/strong&gt; by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
 &lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
@@ -1437,141 +1488,141 @@
 &lt;/table&gt;</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Crowcanyonhome</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="H4" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I4" s="11" t="inlineStr">
+      <c r="I4" s="12" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J4" s="11" t="inlineStr">
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K4" s="11" t="inlineStr">
+      <c r="K4" s="12" t="inlineStr">
         <is>
           <t>CATALINA-SOY-CANDLE--FIXED</t>
         </is>
       </c>
-      <c r="L4" s="11" t="inlineStr">
+      <c r="L4" s="12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M4" s="11" t="inlineStr">
+      <c r="M4" s="12" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N4" s="11" t="inlineStr">
+      <c r="N4" s="12" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O4" s="11" t="inlineStr">
+      <c r="O4" s="12" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P4" s="11" t="inlineStr">
+      <c r="P4" s="12" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q4" s="11" t="inlineStr">
+      <c r="Q4" s="12" t="inlineStr">
         <is>
           <t>24.00</t>
         </is>
       </c>
-      <c r="R4" s="11" t="inlineStr"/>
-      <c r="S4" s="11" t="inlineStr">
+      <c r="R4" s="12" t="inlineStr"/>
+      <c r="S4" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T4" s="11" t="inlineStr">
+      <c r="T4" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U4" s="11" t="inlineStr"/>
-      <c r="V4" s="11" t="inlineStr">
+      <c r="U4" s="12" t="inlineStr"/>
+      <c r="V4" s="12" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0068/3730/5397/files/C121Cgroup2_2.jpg?v=1784043854</t>
         </is>
       </c>
-      <c r="W4" s="11" t="inlineStr">
+      <c r="W4" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X4" s="11" t="inlineStr">
+      <c r="X4" s="12" t="inlineStr">
         <is>
           <t>Catalina Soy Candle 9 oz Mug - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="Y4" s="11" t="inlineStr">
+      <c r="Y4" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z4" s="11" t="inlineStr">
+      <c r="Z4" s="12" t="inlineStr">
         <is>
           <t>Catalina Soy Candle 9 oz Mug | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="AA4" s="11" t="inlineStr">
+      <c r="AA4" s="12" t="inlineStr">
         <is>
           <t>The  Catalina Soy Candle 9 oz Mug  by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engin</t>
         </is>
       </c>
-      <c r="AB4" s="11" t="inlineStr">
+      <c r="AB4" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="AC4" s="11" t="inlineStr">
+      <c r="AC4" s="12" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>cch-stinson-12-mugs</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Stinson Speckle 12 oz Mugs, Set of 4 | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>&lt;p&gt;The &lt;strong&gt;Stinson Speckle 12 oz Mugs, Set of 4&lt;/strong&gt; by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
 &lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
@@ -1586,141 +1637,141 @@
 &lt;/table&gt;</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Crowcanyonhome</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="I5" s="12" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J5" s="11" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
+      <c r="K5" s="12" t="inlineStr">
         <is>
           <t>CCH-STINSON-12-MUGS-FIXED</t>
         </is>
       </c>
-      <c r="L5" s="11" t="inlineStr">
+      <c r="L5" s="12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M5" s="11" t="inlineStr">
+      <c r="M5" s="12" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N5" s="11" t="inlineStr">
+      <c r="N5" s="12" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O5" s="11" t="inlineStr">
+      <c r="O5" s="12" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P5" s="11" t="inlineStr">
+      <c r="P5" s="12" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q5" s="11" t="inlineStr">
+      <c r="Q5" s="12" t="inlineStr">
         <is>
           <t>28.80</t>
         </is>
       </c>
-      <c r="R5" s="11" t="inlineStr"/>
-      <c r="S5" s="11" t="inlineStr">
+      <c r="R5" s="12" t="inlineStr"/>
+      <c r="S5" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T5" s="11" t="inlineStr">
+      <c r="T5" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U5" s="11" t="inlineStr"/>
-      <c r="V5" s="11" t="inlineStr">
+      <c r="U5" s="12" t="inlineStr"/>
+      <c r="V5" s="12" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0068/3730/5397/files/StinsonMugsGroup_3.jpg?v=1779299013</t>
         </is>
       </c>
-      <c r="W5" s="11" t="inlineStr">
+      <c r="W5" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X5" s="11" t="inlineStr">
+      <c r="X5" s="12" t="inlineStr">
         <is>
           <t>Stinson Speckle 12 oz Mugs, Set of 4 - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="Y5" s="11" t="inlineStr">
+      <c r="Y5" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z5" s="11" t="inlineStr">
+      <c r="Z5" s="12" t="inlineStr">
         <is>
           <t>Stinson Speckle 12 oz Mugs, Set of 4 | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="AA5" s="11" t="inlineStr">
+      <c r="AA5" s="12" t="inlineStr">
         <is>
           <t>The  Stinson Speckle 12 oz Mugs, Set of 4  by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtful</t>
         </is>
       </c>
-      <c r="AB5" s="11" t="inlineStr">
+      <c r="AB5" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="AC5" s="11" t="inlineStr">
+      <c r="AC5" s="12" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>cch-vintage-dinner-plates</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Vintage Dinner Plates, Set of 4 | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>&lt;p&gt;The &lt;strong&gt;Vintage Dinner Plates, Set of 4&lt;/strong&gt; by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully engineered to eliminate compromises, it delivers everyday dependability with refined modern aesthetics.&lt;/p&gt;
 &lt;h3&gt;Key Features &amp; Highlights&lt;/h3&gt;
@@ -1735,124 +1786,124 @@
 &lt;/table&gt;</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>Crowcanyonhome</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>Home Goods, Artisanal Design, Heirloom Quality, Handcrafted, Interior Living, Sustainable Home</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="I6" s="12" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>Default Title</t>
         </is>
       </c>
-      <c r="K6" s="11" t="inlineStr">
+      <c r="K6" s="12" t="inlineStr">
         <is>
           <t>CCH-VINTAGE-DINNER-P-FIXED</t>
         </is>
       </c>
-      <c r="L6" s="11" t="inlineStr">
+      <c r="L6" s="12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M6" s="11" t="inlineStr">
+      <c r="M6" s="12" t="inlineStr">
         <is>
           <t>shopify</t>
         </is>
       </c>
-      <c r="N6" s="11" t="inlineStr">
+      <c r="N6" s="12" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="O6" s="11" t="inlineStr">
+      <c r="O6" s="12" t="inlineStr">
         <is>
           <t>deny</t>
         </is>
       </c>
-      <c r="P6" s="11" t="inlineStr">
+      <c r="P6" s="12" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="Q6" s="11" t="inlineStr">
+      <c r="Q6" s="12" t="inlineStr">
         <is>
           <t>48.00</t>
         </is>
       </c>
-      <c r="R6" s="11" t="inlineStr"/>
-      <c r="S6" s="11" t="inlineStr">
+      <c r="R6" s="12" t="inlineStr"/>
+      <c r="S6" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="T6" s="11" t="inlineStr">
+      <c r="T6" s="12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U6" s="11" t="inlineStr"/>
-      <c r="V6" s="11" t="inlineStr">
+      <c r="U6" s="12" t="inlineStr"/>
+      <c r="V6" s="12" t="inlineStr">
         <is>
           <t>https://cdn.shopify.com/s/files/1/0068/3730/5397/files/V20RED-A.jpg?v=1780425866</t>
         </is>
       </c>
-      <c r="W6" s="11" t="inlineStr">
+      <c r="W6" s="12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="X6" s="11" t="inlineStr">
+      <c r="X6" s="12" t="inlineStr">
         <is>
           <t>Vintage Dinner Plates, Set of 4 - Crowcanyonhome Official Product View</t>
         </is>
       </c>
-      <c r="Y6" s="11" t="inlineStr">
+      <c r="Y6" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="Z6" s="11" t="inlineStr">
+      <c r="Z6" s="12" t="inlineStr">
         <is>
           <t>Vintage Dinner Plates, Set of 4 | Handcrafted Artisanal Collection</t>
         </is>
       </c>
-      <c r="AA6" s="11" t="inlineStr">
+      <c r="AA6" s="12" t="inlineStr">
         <is>
           <t>The  Vintage Dinner Plates, Set of 4  by Crowcanyonhome represents the highest standard of intentional craftsmanship and functional design. Thoughtfully en</t>
         </is>
       </c>
-      <c r="AB6" s="11" t="inlineStr">
+      <c r="AB6" s="12" t="inlineStr">
         <is>
           <t>Home &amp; Garden &gt; Kitchen &amp; Dining</t>
         </is>
       </c>
-      <c r="AC6" s="11" t="inlineStr">
+      <c r="AC6" s="12" t="inlineStr">
         <is>
           <t>draft</t>
         </is>

</xml_diff>